<commit_message>
Version final + readme
</commit_message>
<xml_diff>
--- a/pressupost.xlsx
+++ b/pressupost.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ingri\workspace\edd-project-grup-dimecres-dc_g_retrovisors\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B944E8F3-7CEA-421E-B3A1-81D8D614C232}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7071B39-F603-4118-B531-AF996128A529}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{C215AC89-B21C-434C-95CD-7FC53604E0D0}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="124">
   <si>
     <t>#</t>
   </si>
@@ -421,6 +421,9 @@
   </si>
   <si>
     <t>PREU TOTAL (€)</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
   </si>
 </sst>
 </file>
@@ -1832,11 +1835,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3082E9E-407A-4229-90A8-9B20B92E9F5C}">
-  <dimension ref="B1:G6"/>
+  <dimension ref="B1:O6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="2" spans="2:7" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="2" spans="2:15" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B2" s="8" t="s">
         <v>113</v>
       </c>
@@ -1856,7 +1859,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="2:7" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:15" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B3" s="8" t="s">
         <v>119</v>
       </c>
@@ -1875,8 +1878,26 @@
       <c r="G3" s="11">
         <v>842069.8</v>
       </c>
-    </row>
-    <row r="4" spans="2:7" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="J3" t="s">
+        <v>123</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>10</v>
+      </c>
+      <c r="M3">
+        <v>50</v>
+      </c>
+      <c r="N3">
+        <v>1000</v>
+      </c>
+      <c r="O3">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="4" spans="2:15" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B4" s="8" t="s">
         <v>120</v>
       </c>
@@ -1895,8 +1916,26 @@
       <c r="G4" s="11">
         <v>7028.52</v>
       </c>
-    </row>
-    <row r="5" spans="2:7" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="J4" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="K4" s="8">
+        <v>78.97</v>
+      </c>
+      <c r="L4" s="8">
+        <v>639.54</v>
+      </c>
+      <c r="M4" s="8">
+        <v>2913.27</v>
+      </c>
+      <c r="N4" s="8">
+        <v>44071.6</v>
+      </c>
+      <c r="O4" s="9">
+        <v>849098.32</v>
+      </c>
+    </row>
+    <row r="5" spans="2:15" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B5" s="8" t="s">
         <v>121</v>
       </c>
@@ -1916,7 +1955,7 @@
         <v>42.45</v>
       </c>
     </row>
-    <row r="6" spans="2:7" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:15" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B6" s="8" t="s">
         <v>122</v>
       </c>

</xml_diff>